<commit_message>
feat: dialog.xlsx 支援 choice:<node_id> 動態掛載選項，清理 xlsx 表頭/註解冗餘
- scripts/dialog.js 的 buildNpc() 新增 section 欄 choice:<node_id> 語法：
  這種列不必緊接在對應的 node 列後面，可以放在 sheet 任何位置，轉檔時仍會
  依 node_id 掛進該節點的 choices（跟同節點的 choice 列一起依 priority 排
  序）；找不到對應節點只印警告、不中斷轉檔。純粹視覺提醒用的 section 值
  （例如 dynamic）維持原本行為，靜默忽略
- dialog.xlsx：karen/xi 兩個 sheet 拿掉重複的第二個 # 表頭列與中間的
  // 解說註解列（dialog.js 的 splitTables 不靠表格位置分表，只認 section
  欄，兩個表頭內容本來就一樣，拿掉不影響轉檔結果，已重跑腳本驗證輸出
  跟修改前逐位元組相同）；npc_c 這個沒被任何 NPC 用到的空殼 sheet 清空；
  xi 的「關於黑森林討伐」選項改用新的 choice:n_default 語法掛載
- quest.xlsx：xi sheet 的 // 註解列補上原本缺的 conds/actions 欄位標籤
  （純文件性質，parser 本來就略過 // 開頭列，不影響轉檔）
- 同步更新 docs/quest-dialog-architecture.md §1.4 說明新語法

dialog.json/quest.json 重新產生後跟目前版本逐位元組相同，沒有變化。
</commit_message>
<xml_diff>
--- a/xls/quest.xlsx
+++ b/xls/quest.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <workbookPr filterPrivacy="1"/>
   <bookViews>
     <workbookView xWindow="720" yWindow="585" windowWidth="12615" windowHeight="6750" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="karen" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="xi" state="visible" r:id="rId5"/>
+    <sheet name="karen" sheetId="1" r:id="rId1"/>
+    <sheet name="xi" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="50">
   <si>
     <t>//</t>
   </si>
@@ -170,21 +170,28 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="3">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="微軟正黑體 Light"/>
+      <family val="2"/>
       <charset val="136"/>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="12"/>
-      <name val="微軟正黑體 Light"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="新細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -207,13 +214,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999816888943144"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.7999816888943144"/>
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -228,44 +235,78 @@
     </border>
     <border>
       <left/>
-      <right style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -302,7 +343,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -638,9 +679,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="10" style="1" customWidth="1"/>
@@ -652,10 +693,11 @@
     <col min="8" max="8" width="21.5703125" style="1" customWidth="1"/>
     <col min="9" max="9" width="19.7109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="20.28515625" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="31.5" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -682,7 +724,7 @@
       </c>
       <c r="I1" s="4"/>
     </row>
-    <row r="2" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="31.5" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -711,7 +753,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" ht="31.5" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="31.5" customHeight="1">
       <c r="B3" s="5" t="s">
         <v>15</v>
       </c>
@@ -733,7 +775,7 @@
       </c>
       <c r="I3" s="6"/>
     </row>
-    <row r="5" ht="31.5" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="31.5" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -765,7 +807,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" ht="31.5" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="31.5" customHeight="1">
       <c r="B6" s="7" t="s">
         <v>15</v>
       </c>
@@ -788,7 +830,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" ht="31.5" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="31.5" customHeight="1">
       <c r="B7" s="7" t="s">
         <v>15</v>
       </c>
@@ -813,7 +855,7 @@
       </c>
       <c r="J7" s="8"/>
     </row>
-    <row r="8" ht="15.75" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="15.75" customHeight="1">
       <c r="B8" s="7" t="s">
         <v>15</v>
       </c>
@@ -838,7 +880,7 @@
       </c>
       <c r="J8" s="8"/>
     </row>
-    <row r="9" ht="15.75" customHeight="1" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="15.75" customHeight="1">
       <c r="B9" s="9" t="s">
         <v>15</v>
       </c>
@@ -860,15 +902,16 @@
       <c r="J9" s="10"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -882,7 +925,7 @@
     <col min="10" max="10" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="31.5" customHeight="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -907,8 +950,14 @@
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="31.5" customHeight="1">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -937,7 +986,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" ht="47.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="47.25" customHeight="1">
       <c r="B3" s="5" t="s">
         <v>37</v>
       </c>
@@ -963,8 +1012,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="31.5" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="31.5" customHeight="1">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -996,7 +1044,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" ht="31.5" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="31.5" customHeight="1">
       <c r="B6" s="7" t="s">
         <v>37</v>
       </c>
@@ -1019,7 +1067,7 @@
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="15.75" customHeight="1">
       <c r="B7" s="7" t="s">
         <v>37</v>
       </c>
@@ -1044,7 +1092,7 @@
       </c>
       <c r="J7" s="8"/>
     </row>
-    <row r="8" ht="31.5" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="31.5" customHeight="1">
       <c r="B8" s="7" t="s">
         <v>37</v>
       </c>
@@ -1067,7 +1115,7 @@
       </c>
       <c r="J8" s="8"/>
     </row>
-    <row r="9" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="15.75" customHeight="1">
       <c r="B9" s="9" t="s">
         <v>37</v>
       </c>
@@ -1089,7 +1137,8 @@
       <c r="J9" s="10"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>